<commit_message>
Atualização do roadmap com novas empresas
</commit_message>
<xml_diff>
--- a/existing-spreadsheets/road_map_table_EN.xlsx
+++ b/existing-spreadsheets/road_map_table_EN.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="info" sheetId="1" r:id="R8cf1b9664eca4207"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grouped" sheetId="2" r:id="R5f6f656ffefc4257"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="info" sheetId="1" r:id="R400128010c4041e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="grouped" sheetId="2" r:id="R1956f2944522442d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="17">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF000000"/>
@@ -96,8 +96,17 @@
       <x:color rgb="FF000000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:color theme="1"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -159,8 +168,23 @@
         <x:fgColor rgb="FFF3F3F3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F1F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9D9D9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="21">
+  <x:borders count="23">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -376,11 +400,39 @@
         <x:color indexed="1" rgb="FF000000"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF222222"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF222222"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF222222"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF222222"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF444444"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FF444444"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF444444"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF444444"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="240">
+  <x:cellXfs count="280">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -1092,6 +1144,126 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="16" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="13" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="14" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="14" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="15" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="14" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1143,9 +1315,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2825,17 +2997,73 @@
         <x:v>https://www.gov.br/inpe/pt-br</x:v>
       </x:c>
     </x:row>
-    <x:row r="50" ht="15.75" customHeight="1">
-      <x:c r="C50" s="17"/>
-    </x:row>
-    <x:row r="51" ht="15.75" customHeight="1">
-      <x:c r="C51" s="17"/>
-    </x:row>
-    <x:row r="52" ht="15.75" customHeight="1">
-      <x:c r="C52" s="17"/>
-    </x:row>
-    <x:row r="53" ht="15.75" customHeight="1">
-      <x:c r="C53" s="17"/>
+    <x:row r="50" ht="53" customHeight="1">
+      <x:c r="A50" s="262" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B50" s="262" t="str">
+        <x:v>AEL Sistemas</x:v>
+      </x:c>
+      <x:c r="C50" s="264" t="str">
+        <x:v>Development, integration and production of advanced electronics, avionics, radar and defense systems; specific in-house FPGA/RTL activities are not confirmed by the cited source.</x:v>
+      </x:c>
+      <x:c r="D50" s="262" t="str">
+        <x:v>Private company (Brazilian)</x:v>
+      </x:c>
+      <x:c r="E50" s="279" t="str">
+        <x:v>https://www.ael.com.br/sobre-nos/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="53" customHeight="1">
+      <x:c r="A51" s="262" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B51" s="262" t="str">
+        <x:v>Grupo Tellescom</x:v>
+      </x:c>
+      <x:c r="C51" s="264" t="str">
+        <x:v>Planned semiconductor assembly, packaging and test facility in Cachoeirinha (RS), with automotive, wireless communications and IoT applications; not yet an operating plant.</x:v>
+      </x:c>
+      <x:c r="D51" s="262" t="str">
+        <x:v>Private company (Brazilian)</x:v>
+      </x:c>
+      <x:c r="E51" s="279" t="str">
+        <x:v>https://tellescom.com.br/tellescom-mantem-projeto-para-instalar-fabrica-de-chips-de-r-1-bilhao-em-cachoeirinha/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="53" customHeight="1">
+      <x:c r="A52" s="262" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B52" s="262" t="str">
+        <x:v>OSIRIS</x:v>
+      </x:c>
+      <x:c r="C52" s="264" t="str">
+        <x:v>Nonprofit open-source RISC-V research group developing digital integrated circuits, soft IP, SoCs and ASICs, with an emphasis on VLSI design.</x:v>
+      </x:c>
+      <x:c r="D52" s="262" t="str">
+        <x:v>Nonprofit research group</x:v>
+      </x:c>
+      <x:c r="E52" s="279" t="str">
+        <x:v>https://www.osirisgroup.com.br/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="53" customHeight="1">
+      <x:c r="A53" s="262" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B53" s="262" t="str">
+        <x:v>Instituto SENAI (RS)</x:v>
+      </x:c>
+      <x:c r="C53" s="264" t="str">
+        <x:v>SENAI-RS applied R&amp;D in industrial electronics, sensor systems, embedded technologies and artificial intelligence; FPGA/IC design at the cited institute is not specifically confirmed.</x:v>
+      </x:c>
+      <x:c r="D53" s="262" t="str">
+        <x:v>Private nonprofit research center</x:v>
+      </x:c>
+      <x:c r="E53" s="279" t="str">
+        <x:v>https://www.senairs.org.br/institutos/sistemas-de-sensoriamento</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="15.75" customHeight="1">
       <x:c r="C54" s="17"/>
@@ -4156,635 +4384,651 @@
     <x:col min="3" max="6" width="12.630000114440918" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="24" customHeight="1">
-      <x:c r="A1" s="231" t="str">
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="257" t="str">
         <x:v>No.</x:v>
       </x:c>
-      <x:c r="B1" s="231" t="str">
+      <x:c r="B1" s="257" t="str">
         <x:v>Company</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="235" t="str">
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="256" t="str">
         <x:v>Manaus</x:v>
       </x:c>
-      <x:c r="B2" s="236"/>
-    </x:row>
-    <x:row r="3" ht="20" customHeight="1">
-      <x:c r="A3" s="239" t="n">
+      <x:c r="B2" s="256"/>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="253" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B3" s="239" t="str">
+      <x:c r="B3" s="253" t="str">
         <x:v>Instituto SENAI de Inovação em Microeletrônica</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="20" customHeight="1">
-      <x:c r="A4" s="239" t="n">
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="253" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B4" s="239" t="str">
+      <x:c r="B4" s="253" t="str">
         <x:v>ADATA</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="20" customHeight="1">
-      <x:c r="A5" s="239" t="n">
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="253" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B5" s="239" t="str">
+      <x:c r="B5" s="253" t="str">
         <x:v>Zilia</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="20" customHeight="1">
-      <x:c r="A6" s="239" t="n">
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="253" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B6" s="239" t="str">
+      <x:c r="B6" s="253" t="str">
         <x:v>Stoneridge</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="20" customHeight="1">
-      <x:c r="A7" s="239" t="n">
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="253" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B7" s="239" t="str">
+      <x:c r="B7" s="253" t="str">
         <x:v>HBR</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="20" customHeight="1">
-      <x:c r="A8" s="239" t="n">
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="253" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B8" s="239" t="str">
+      <x:c r="B8" s="253" t="str">
         <x:v>Instituto de Pesquisas ELDORADO</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="20" customHeight="1">
-      <x:c r="A9" s="239" t="n">
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="253" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B9" s="239" t="str">
+      <x:c r="B9" s="253" t="str">
         <x:v>HT Micron</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="20" customHeight="1">
-      <x:c r="A10" s="239" t="n">
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="253" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B10" s="239" t="str">
+      <x:c r="B10" s="253" t="str">
         <x:v>CCBS / TERA</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="235" t="str">
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="256" t="str">
         <x:v>Brasília</x:v>
       </x:c>
-      <x:c r="B11" s="236"/>
-    </x:row>
-    <x:row r="12" ht="20" customHeight="1">
-      <x:c r="A12" s="239" t="n">
+      <x:c r="B11" s="256"/>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="253" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B12" s="239" t="str">
+      <x:c r="B12" s="253" t="str">
         <x:v>HBR</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="20" customHeight="1">
-      <x:c r="A13" s="239" t="n">
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="253" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B13" s="239" t="str">
+      <x:c r="B13" s="253" t="str">
         <x:v>Instituto de Pesquisas ELDORADO</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="237" t="str">
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" s="256" t="str">
         <x:v>Campina Grande</x:v>
       </x:c>
-      <x:c r="B14" s="238"/>
-    </x:row>
-    <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="239" t="n">
+      <x:c r="B14" s="256"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="253" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="B15" s="239" t="str">
+      <x:c r="B15" s="253" t="str">
         <x:v>HWiT</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="237" t="str">
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="A16" s="256" t="str">
         <x:v>Salvador</x:v>
       </x:c>
-      <x:c r="B16" s="238"/>
-    </x:row>
-    <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="239" t="n">
+      <x:c r="B16" s="256"/>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="253" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B17" s="239" t="str">
+      <x:c r="B17" s="253" t="str">
         <x:v>SENAI CIMATEC</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="20" customHeight="1">
-      <x:c r="A18" s="239" t="n">
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="253" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="B18" s="239" t="str">
+      <x:c r="B18" s="253" t="str">
         <x:v>HBR</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="237" t="str">
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="256" t="str">
         <x:v>Minas Gerais State Interior</x:v>
       </x:c>
-      <x:c r="B19" s="238"/>
-    </x:row>
-    <x:row r="20" ht="20" customHeight="1">
-      <x:c r="A20" s="239" t="n">
+      <x:c r="B19" s="256"/>
+    </x:row>
+    <x:row r="20" ht="24" customHeight="1">
+      <x:c r="A20" s="253" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B20" s="239" t="str">
+      <x:c r="B20" s="253" t="str">
         <x:v>LC-e</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="20" customHeight="1">
-      <x:c r="A21" s="239" t="n">
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="253" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="B21" s="239" t="str">
+      <x:c r="B21" s="253" t="str">
         <x:v>Inatel</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="20" customHeight="1">
-      <x:c r="A22" s="239" t="n">
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="253" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="B22" s="239" t="str">
+      <x:c r="B22" s="253" t="str">
         <x:v>Modirum | GESPI</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="20" customHeight="1">
-      <x:c r="A23" s="239" t="n">
+    <x:row r="23" ht="24" customHeight="1">
+      <x:c r="A23" s="253" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="B23" s="239" t="str">
+      <x:c r="B23" s="253" t="str">
         <x:v>Marelli</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="20" customHeight="1">
-      <x:c r="A24" s="239" t="n">
+    <x:row r="24" ht="24" customHeight="1">
+      <x:c r="A24" s="253" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B24" s="239" t="str">
+      <x:c r="B24" s="253" t="str">
         <x:v>Stellantis</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="20" customHeight="1">
-      <x:c r="A25" s="239" t="n">
+    <x:row r="25" ht="24" customHeight="1">
+      <x:c r="A25" s="253" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="B25" s="239" t="str">
+      <x:c r="B25" s="253" t="str">
         <x:v>Multilaser</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="24" customHeight="1">
-      <x:c r="A26" s="237" t="str">
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="A26" s="256" t="str">
         <x:v>Belo Horizonte and Surrounding Area</x:v>
       </x:c>
-      <x:c r="B26" s="238"/>
-    </x:row>
-    <x:row r="27" ht="20" customHeight="1">
-      <x:c r="A27" s="239" t="n">
+      <x:c r="B26" s="256"/>
+    </x:row>
+    <x:row r="27" ht="24" customHeight="1">
+      <x:c r="A27" s="253" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="B27" s="239" t="str">
+      <x:c r="B27" s="253" t="str">
         <x:v>Cadence</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="20" customHeight="1">
-      <x:c r="A28" s="239" t="n">
+    <x:row r="28" ht="24" customHeight="1">
+      <x:c r="A28" s="253" t="n">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B28" s="239" t="str">
+      <x:c r="B28" s="253" t="str">
         <x:v>RFIDO Design</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="24" customHeight="1">
-      <x:c r="A29" s="237" t="str">
+    <x:row r="29" ht="28" customHeight="1">
+      <x:c r="A29" s="256" t="str">
         <x:v>Campinas and Surrounding Area</x:v>
       </x:c>
-      <x:c r="B29" s="238"/>
-    </x:row>
-    <x:row r="30" ht="20" customHeight="1">
-      <x:c r="A30" s="239" t="n">
+      <x:c r="B29" s="256"/>
+    </x:row>
+    <x:row r="30" ht="24" customHeight="1">
+      <x:c r="A30" s="253" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B30" s="239" t="str">
+      <x:c r="B30" s="253" t="str">
         <x:v>Von Braun Labs</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="20" customHeight="1">
-      <x:c r="A31" s="239" t="n">
+    <x:row r="31" ht="24" customHeight="1">
+      <x:c r="A31" s="253" t="n">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B31" s="239" t="str">
+      <x:c r="B31" s="253" t="str">
         <x:v>ADATA</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="20" customHeight="1">
-      <x:c r="A32" s="239" t="n">
+    <x:row r="32" ht="24" customHeight="1">
+      <x:c r="A32" s="253" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B32" s="239" t="str">
+      <x:c r="B32" s="253" t="str">
         <x:v>HBR</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="20" customHeight="1">
-      <x:c r="A33" s="239" t="n">
+    <x:row r="33" ht="24" customHeight="1">
+      <x:c r="A33" s="253" t="n">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="B33" s="239" t="str">
+      <x:c r="B33" s="253" t="str">
         <x:v>HWiT</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="20" customHeight="1">
-      <x:c r="A34" s="239" t="n">
+    <x:row r="34" ht="24" customHeight="1">
+      <x:c r="A34" s="253" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="B34" s="239" t="str">
+      <x:c r="B34" s="253" t="str">
         <x:v>EnSilica</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="20" customHeight="1">
-      <x:c r="A35" s="239" t="n">
+    <x:row r="35" ht="24" customHeight="1">
+      <x:c r="A35" s="253" t="n">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="B35" s="239" t="str">
+      <x:c r="B35" s="253" t="str">
         <x:v>CPQD</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="20" customHeight="1">
-      <x:c r="A36" s="239" t="n">
+    <x:row r="36" ht="24" customHeight="1">
+      <x:c r="A36" s="253" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="B36" s="239" t="str">
+      <x:c r="B36" s="253" t="str">
         <x:v>Aedvices</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="20" customHeight="1">
-      <x:c r="A37" s="239" t="n">
+    <x:row r="37" ht="24" customHeight="1">
+      <x:c r="A37" s="253" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B37" s="239" t="str">
+      <x:c r="B37" s="253" t="str">
         <x:v>Instituto de Pesquisas ELDORADO</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="20" customHeight="1">
-      <x:c r="A38" s="239" t="n">
+    <x:row r="38" ht="24" customHeight="1">
+      <x:c r="A38" s="253" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B38" s="239" t="str">
+      <x:c r="B38" s="253" t="str">
         <x:v>Stoneridge</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="20" customHeight="1">
-      <x:c r="A39" s="239" t="n">
+    <x:row r="39" ht="24" customHeight="1">
+      <x:c r="A39" s="253" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B39" s="239" t="str">
+      <x:c r="B39" s="253" t="str">
         <x:v>Valeo</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="20" customHeight="1">
-      <x:c r="A40" s="239" t="n">
+    <x:row r="40" ht="24" customHeight="1">
+      <x:c r="A40" s="253" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="B40" s="239" t="str">
+      <x:c r="B40" s="253" t="str">
         <x:v>Cadence</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="20" customHeight="1">
-      <x:c r="A41" s="239" t="n">
+    <x:row r="41" ht="24" customHeight="1">
+      <x:c r="A41" s="253" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B41" s="239" t="str">
+      <x:c r="B41" s="253" t="str">
         <x:v>CNPEM</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="20" customHeight="1">
-      <x:c r="A42" s="239" t="n">
+    <x:row r="42" ht="24" customHeight="1">
+      <x:c r="A42" s="253" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="B42" s="239" t="str">
+      <x:c r="B42" s="253" t="str">
         <x:v>CTI Renato Archer</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="20" customHeight="1">
-      <x:c r="A43" s="239" t="n">
+    <x:row r="43" ht="24" customHeight="1">
+      <x:c r="A43" s="253" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="B43" s="239" t="str">
+      <x:c r="B43" s="253" t="str">
         <x:v>HCLTech</x:v>
       </x:c>
     </x:row>
-    <x:row r="44" ht="24" customHeight="1">
-      <x:c r="A44" s="235" t="str">
+    <x:row r="44" ht="28" customHeight="1">
+      <x:c r="A44" s="256" t="str">
         <x:v>Florianópolis</x:v>
       </x:c>
-      <x:c r="B44" s="236"/>
-    </x:row>
-    <x:row r="45" ht="20" customHeight="1">
-      <x:c r="A45" s="239" t="n">
+      <x:c r="B44" s="256"/>
+    </x:row>
+    <x:row r="45" ht="24" customHeight="1">
+      <x:c r="A45" s="253" t="n">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B45" s="239" t="str">
+      <x:c r="B45" s="253" t="str">
         <x:v>Macnica DHW</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="20" customHeight="1">
-      <x:c r="A46" s="239" t="n">
+    <x:row r="46" ht="24" customHeight="1">
+      <x:c r="A46" s="253" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B46" s="239" t="str">
+      <x:c r="B46" s="253" t="str">
+        <x:v>Chipus</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="24" customHeight="1">
+      <x:c r="A47" s="253" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B47" s="253" t="str">
+        <x:v>Synopsys</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="24" customHeight="1">
+      <x:c r="A48" s="253" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B48" s="253" t="str">
+        <x:v>OSIRIS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="24" customHeight="1">
+      <x:c r="A49" s="253" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B49" s="253" t="str">
         <x:v>Silicium</x:v>
       </x:c>
     </x:row>
-    <x:row r="47" ht="20" customHeight="1">
-      <x:c r="A47" s="239" t="n">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B47" s="239" t="str">
-        <x:v>Chipus</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="20" customHeight="1">
-      <x:c r="A48" s="239" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="B48" s="239" t="str">
-        <x:v>Synopsys</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49" ht="24" customHeight="1">
-      <x:c r="A49" s="237" t="str">
+    <x:row r="50" ht="28" customHeight="1">
+      <x:c r="A50" s="256" t="str">
         <x:v>Porto Alegre and Surrounding Area</x:v>
       </x:c>
-      <x:c r="B49" s="238"/>
-    </x:row>
-    <x:row r="50" ht="20" customHeight="1">
-      <x:c r="A50" s="239" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="B50" s="239" t="str">
+      <x:c r="B50" s="256"/>
+    </x:row>
+    <x:row r="51" ht="24" customHeight="1">
+      <x:c r="A51" s="253" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B51" s="253" t="str">
+        <x:v>Impinj</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="24" customHeight="1">
+      <x:c r="A52" s="253" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B52" s="253" t="str">
+        <x:v>SILVACO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="24" customHeight="1">
+      <x:c r="A53" s="253" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B53" s="253" t="str">
+        <x:v>HCLTech</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="24" customHeight="1">
+      <x:c r="A54" s="253" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B54" s="253" t="str">
+        <x:v>AEL Sistemas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="24" customHeight="1">
+      <x:c r="A55" s="253" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B55" s="253" t="str">
+        <x:v>Grupo Tellescom</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="24" customHeight="1">
+      <x:c r="A56" s="253" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B56" s="253" t="str">
+        <x:v>Valeo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="24" customHeight="1">
+      <x:c r="A57" s="253" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B57" s="253" t="str">
+        <x:v>Instituto de Pesquisas ELDORADO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="24" customHeight="1">
+      <x:c r="A58" s="253" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B58" s="253" t="str">
+        <x:v>EnSilica</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="24" customHeight="1">
+      <x:c r="A59" s="253" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B59" s="253" t="str">
+        <x:v>itt Chip — Unisinos</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="24" customHeight="1">
+      <x:c r="A60" s="253" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B60" s="253" t="str">
+        <x:v>CEITEC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="24" customHeight="1">
+      <x:c r="A61" s="253" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B61" s="253" t="str">
+        <x:v>Instituto SENAI (RS)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="24" customHeight="1">
+      <x:c r="A62" s="253" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B62" s="253" t="str">
+        <x:v>InPlace</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="24" customHeight="1">
+      <x:c r="A63" s="253" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B63" s="253" t="str">
         <x:v>HT Micron</x:v>
       </x:c>
     </x:row>
-    <x:row r="51" ht="20" customHeight="1">
-      <x:c r="A51" s="239" t="n">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B51" s="239" t="str">
-        <x:v>Impinj</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="20" customHeight="1">
-      <x:c r="A52" s="239" t="n">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B52" s="239" t="str">
-        <x:v>SILVACO</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="20" customHeight="1">
-      <x:c r="A53" s="239" t="n">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="B53" s="239" t="str">
+    <x:row r="64" ht="28" customHeight="1">
+      <x:c r="A64" s="256" t="str">
+        <x:v>São Paulo State Interior</x:v>
+      </x:c>
+      <x:c r="B64" s="256"/>
+    </x:row>
+    <x:row r="65" ht="24" customHeight="1">
+      <x:c r="A65" s="253" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B65" s="253" t="str">
+        <x:v>Macnica DHW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="24" customHeight="1">
+      <x:c r="A66" s="253" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B66" s="253" t="str">
+        <x:v>WG3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="24" customHeight="1">
+      <x:c r="A67" s="253" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B67" s="253" t="str">
+        <x:v>Chip Inventor</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="24" customHeight="1">
+      <x:c r="A68" s="253" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B68" s="253" t="str">
+        <x:v>Beontag</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="24" customHeight="1">
+      <x:c r="A69" s="253" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B69" s="253" t="str">
+        <x:v>SPICTEC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="24" customHeight="1">
+      <x:c r="A70" s="253" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B70" s="253" t="str">
+        <x:v>LSI-TEC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="28" customHeight="1">
+      <x:c r="A71" s="256" t="str">
+        <x:v>Curitiba and Surrounding Area</x:v>
+      </x:c>
+      <x:c r="B71" s="256"/>
+    </x:row>
+    <x:row r="72" ht="24" customHeight="1">
+      <x:c r="A72" s="253" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B72" s="253" t="str">
         <x:v>HCLTech</x:v>
       </x:c>
     </x:row>
-    <x:row r="54" ht="20" customHeight="1">
-      <x:c r="A54" s="239" t="n">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="B54" s="239" t="str">
-        <x:v>Valeo</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55" ht="20" customHeight="1">
-      <x:c r="A55" s="239" t="n">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="B55" s="239" t="str">
-        <x:v>Instituto de Pesquisas ELDORADO</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="20" customHeight="1">
-      <x:c r="A56" s="239" t="n">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="B56" s="239" t="str">
-        <x:v>EnSilica</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57" ht="20" customHeight="1">
-      <x:c r="A57" s="239" t="n">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B57" s="239" t="str">
-        <x:v>itt Chip — Unisinos</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58" ht="20" customHeight="1">
-      <x:c r="A58" s="239" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="B58" s="239" t="str">
-        <x:v>CEITEC</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59" ht="20" customHeight="1">
-      <x:c r="A59" s="239" t="n">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="B59" s="239" t="str">
-        <x:v>InPlace</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="24" customHeight="1">
-      <x:c r="A60" s="235" t="str">
-        <x:v>São Paulo State Interior</x:v>
-      </x:c>
-      <x:c r="B60" s="236"/>
-    </x:row>
-    <x:row r="61" ht="20" customHeight="1">
-      <x:c r="A61" s="239" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="B61" s="239" t="str">
-        <x:v>LSI-TEC</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62" ht="20" customHeight="1">
-      <x:c r="A62" s="239" t="n">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="B62" s="239" t="str">
-        <x:v>Macnica DHW</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="20" customHeight="1">
-      <x:c r="A63" s="239" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="B63" s="239" t="str">
-        <x:v>WG3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64" ht="20" customHeight="1">
-      <x:c r="A64" s="239" t="n">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="B64" s="239" t="str">
-        <x:v>Chip Inventor</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" ht="20" customHeight="1">
-      <x:c r="A65" s="239" t="n">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="B65" s="239" t="str">
-        <x:v>Beontag</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="20" customHeight="1">
-      <x:c r="A66" s="239" t="n">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="B66" s="239" t="str">
-        <x:v>SPICTEC</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="24" customHeight="1">
-      <x:c r="A67" s="235" t="str">
-        <x:v>Curitiba and Surrounding Area</x:v>
-      </x:c>
-      <x:c r="B67" s="236"/>
-    </x:row>
-    <x:row r="68" ht="20" customHeight="1">
-      <x:c r="A68" s="239" t="n">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="B68" s="239" t="str">
+    <x:row r="73" ht="24" customHeight="1">
+      <x:c r="A73" s="253" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B73" s="253" t="str">
         <x:v>Thales Group</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" ht="20" customHeight="1">
-      <x:c r="A69" s="239" t="n">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="B69" s="239" t="str">
-        <x:v>HCLTech</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70" ht="24" customHeight="1">
-      <x:c r="A70" s="235" t="str">
+    <x:row r="74" ht="28" customHeight="1">
+      <x:c r="A74" s="256" t="str">
         <x:v>Rio Grande do Sul State Interior</x:v>
       </x:c>
-      <x:c r="B70" s="236"/>
-    </x:row>
-    <x:row r="71" ht="20" customHeight="1">
-      <x:c r="A71" s="239" t="n">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="B71" s="239" t="str">
+      <x:c r="B74" s="256"/>
+    </x:row>
+    <x:row r="75" ht="24" customHeight="1">
+      <x:c r="A75" s="253" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B75" s="253" t="str">
+        <x:v>TUNA Semicondutores</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="24" customHeight="1">
+      <x:c r="A76" s="253" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B76" s="253" t="str">
         <x:v>GMicro UFSM</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" ht="20" customHeight="1">
-      <x:c r="A72" s="239" t="n">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="B72" s="239" t="str">
-        <x:v>TUNA Semicondutores</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="24" customHeight="1">
-      <x:c r="A73" s="235" t="str">
+    <x:row r="77" ht="28" customHeight="1">
+      <x:c r="A77" s="256" t="str">
         <x:v>São José dos Campos and Surrounding Area</x:v>
       </x:c>
-      <x:c r="B73" s="236"/>
-    </x:row>
-    <x:row r="74" ht="20" customHeight="1">
-      <x:c r="A74" s="239" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B74" s="239" t="str">
+      <x:c r="B77" s="256"/>
+    </x:row>
+    <x:row r="78" ht="24" customHeight="1">
+      <x:c r="A78" s="253" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B78" s="253" t="str">
+        <x:v>Boeing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="24" customHeight="1">
+      <x:c r="A79" s="253" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B79" s="253" t="str">
+        <x:v>Embraer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="24" customHeight="1">
+      <x:c r="A80" s="253" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B80" s="253" t="str">
+        <x:v>Thales Group</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="24" customHeight="1">
+      <x:c r="A81" s="254" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B81" s="254" t="str">
         <x:v>SIATT</x:v>
       </x:c>
     </x:row>
-    <x:row r="75" ht="20" customHeight="1">
-      <x:c r="A75" s="239" t="n">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B75" s="239" t="str">
+    <x:row r="82" ht="24" customHeight="1">
+      <x:c r="A82" s="254" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B82" s="254" t="str">
         <x:v>IACIT</x:v>
       </x:c>
     </x:row>
-    <x:row r="76" ht="20" customHeight="1">
-      <x:c r="A76" s="239" t="n">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="B76" s="239" t="str">
+    <x:row r="83" ht="24" customHeight="1">
+      <x:c r="A83" s="254" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B83" s="254" t="str">
         <x:v>INPE</x:v>
       </x:c>
     </x:row>
-    <x:row r="77" ht="20" customHeight="1">
-      <x:c r="A77" s="239" t="n">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="B77" s="239" t="str">
+    <x:row r="84" ht="24" customHeight="1">
+      <x:c r="A84" s="254" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="B84" s="254" t="str">
         <x:v>Modirum | GESPI</x:v>
       </x:c>
-    </x:row>
-    <x:row r="78" ht="20" customHeight="1">
-      <x:c r="A78" s="239" t="n">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="B78" s="239" t="str">
-        <x:v>Boeing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="79" ht="20" customHeight="1">
-      <x:c r="A79" s="239" t="n">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="B79" s="239" t="str">
-        <x:v>Embraer</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="80" ht="20" customHeight="1">
-      <x:c r="A80" s="239" t="n">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="B80" s="239" t="str">
-        <x:v>Thales Group</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="81" ht="15.75" customHeight="1">
-      <x:c r="A81" s="20"/>
-      <x:c r="B81" s="20"/>
-    </x:row>
-    <x:row r="82" ht="15.75" customHeight="1">
-      <x:c r="A82" s="20"/>
-      <x:c r="B82" s="20"/>
-    </x:row>
-    <x:row r="83" ht="15.75" customHeight="1">
-      <x:c r="A83" s="20"/>
-      <x:c r="B83" s="20"/>
-    </x:row>
-    <x:row r="84" ht="15.75" customHeight="1">
-      <x:c r="A84" s="20"/>
-      <x:c r="B84" s="20"/>
     </x:row>
     <x:row r="85" ht="15.75" customHeight="1">
       <x:c r="A85" s="20"/>
@@ -6246,11 +6490,11 @@
     <x:mergeCell ref="A26:B26"/>
     <x:mergeCell ref="A29:B29"/>
     <x:mergeCell ref="A44:B44"/>
-    <x:mergeCell ref="A49:B49"/>
-    <x:mergeCell ref="A60:B60"/>
-    <x:mergeCell ref="A67:B67"/>
-    <x:mergeCell ref="A70:B70"/>
-    <x:mergeCell ref="A73:B73"/>
+    <x:mergeCell ref="A50:B50"/>
+    <x:mergeCell ref="A64:B64"/>
+    <x:mergeCell ref="A71:B71"/>
+    <x:mergeCell ref="A74:B74"/>
+    <x:mergeCell ref="A77:B77"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>